<commit_message>
archivo definitivo para N definido por Swap con ambos criterios independientes
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_NEH(SwapFirstImprovement).xlsx
+++ b/code/resultados/NWJSSP_OADG_NEH(SwapFirstImprovement).xlsx
@@ -472,7 +472,7 @@
         <v>6786530</v>
       </c>
       <c r="B1" t="n">
-        <v>176301</v>
+        <v>208178</v>
       </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
@@ -936,7 +936,7 @@
         <v>10384</v>
       </c>
       <c r="B1" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2">
@@ -990,7 +990,7 @@
         <v>11692</v>
       </c>
       <c r="B1" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -1044,7 +1044,7 @@
         <v>19770</v>
       </c>
       <c r="B1" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2">
@@ -1128,7 +1128,7 @@
         <v>20507</v>
       </c>
       <c r="B1" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2">
@@ -1212,7 +1212,7 @@
         <v>111153</v>
       </c>
       <c r="B1" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2">
@@ -1320,7 +1320,7 @@
         <v>6926870</v>
       </c>
       <c r="B1" t="n">
-        <v>56459</v>
+        <v>55486</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
cleaning and preparing for last run
</commit_message>
<xml_diff>
--- a/code/resultados/NWJSSP_OADG_NEH(SwapFirstImprovement).xlsx
+++ b/code/resultados/NWJSSP_OADG_NEH(SwapFirstImprovement).xlsx
@@ -14,6 +14,8 @@
     <sheet name="ft20r" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="tai_j10_m10_1" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="tai_j10_m10_1r" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="tai_j100_m100_1" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="tai_j100_m100_1r" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -424,7 +426,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>309</v>
+        <v>320</v>
       </c>
       <c r="B1" t="n">
         <v>3</v>
@@ -432,22 +434,346 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2" t="n">
         <v>0</v>
       </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CV2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>43676166</v>
+      </c>
+      <c r="B1" t="n">
+        <v>3628088</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>63399</v>
+      </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>743061</v>
       </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>432713</v>
       </c>
       <c r="D2" t="n">
-        <v>36</v>
+        <v>98110</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>55144</v>
       </c>
       <c r="F2" t="n">
-        <v>43</v>
+        <v>306907</v>
+      </c>
+      <c r="G2" t="n">
+        <v>823951</v>
+      </c>
+      <c r="H2" t="n">
+        <v>643203</v>
+      </c>
+      <c r="I2" t="n">
+        <v>95858</v>
+      </c>
+      <c r="J2" t="n">
+        <v>256466</v>
+      </c>
+      <c r="K2" t="n">
+        <v>835858</v>
+      </c>
+      <c r="L2" t="n">
+        <v>311706</v>
+      </c>
+      <c r="M2" t="n">
+        <v>497458</v>
+      </c>
+      <c r="N2" t="n">
+        <v>648106</v>
+      </c>
+      <c r="O2" t="n">
+        <v>627283</v>
+      </c>
+      <c r="P2" t="n">
+        <v>472871</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>293217</v>
+      </c>
+      <c r="R2" t="n">
+        <v>267858</v>
+      </c>
+      <c r="S2" t="n">
+        <v>575981</v>
+      </c>
+      <c r="T2" t="n">
+        <v>159742</v>
+      </c>
+      <c r="U2" t="n">
+        <v>42097</v>
+      </c>
+      <c r="V2" t="n">
+        <v>837137</v>
+      </c>
+      <c r="W2" t="n">
+        <v>290527</v>
+      </c>
+      <c r="X2" t="n">
+        <v>233860</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>90341</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>491702</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>701525</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>407122</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>791501</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>751043</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>563092</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>359570</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>484681</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>590775</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>146332</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>669893</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>151978</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>368094</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>242073</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>377046</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>139562</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>705</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>330093</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>271206</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>712088</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>3102</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>21013</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>480034</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>92765</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>188184</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>303741</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>601339</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>251228</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>397117</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>214578</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>165914</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>12994</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>753437</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>199103</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>349509</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>624383</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>464821</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>780535</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>186995</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>66036</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>410115</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>149421</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>435299</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>555746</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>64661</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>450540</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>584483</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>206096</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>723315</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>785380</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>16033</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>131092</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>589182</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>428507</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>118863</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>663712</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>511838</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>22017</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>128971</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>250553</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>60932</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>323868</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>525123</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>534830</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>652196</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>535259</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>202111</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>699425</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>784333</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>722252</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>360524</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>455954</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>370648</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>814456</v>
       </c>
     </row>
   </sheetData>
@@ -466,7 +792,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>324</v>
+        <v>349</v>
       </c>
       <c r="B1" t="n">
         <v>1</v>
@@ -474,22 +800,22 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="n">
-        <v>19</v>
-      </c>
       <c r="C2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="F2" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -508,10 +834,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>10384</v>
+        <v>10031</v>
       </c>
       <c r="B1" t="n">
-        <v>19</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2">
@@ -519,31 +845,31 @@
         <v>46</v>
       </c>
       <c r="B2" t="n">
-        <v>132</v>
+        <v>201</v>
       </c>
       <c r="C2" t="n">
-        <v>509</v>
+        <v>776</v>
       </c>
       <c r="D2" t="n">
-        <v>1281</v>
+        <v>360</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1057</v>
+        <v>1079</v>
       </c>
       <c r="G2" t="n">
-        <v>463</v>
+        <v>561</v>
       </c>
       <c r="H2" t="n">
-        <v>840</v>
+        <v>613</v>
       </c>
       <c r="I2" t="n">
-        <v>693</v>
+        <v>84</v>
       </c>
       <c r="J2" t="n">
-        <v>254</v>
+        <v>1202</v>
       </c>
     </row>
   </sheetData>
@@ -562,42 +888,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>11692</v>
+        <v>10378</v>
       </c>
       <c r="B1" t="n">
-        <v>14</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>658</v>
+        <v>299</v>
       </c>
       <c r="B2" t="n">
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>380</v>
+        <v>811</v>
       </c>
       <c r="D2" t="n">
-        <v>1142</v>
+        <v>1265</v>
       </c>
       <c r="E2" t="n">
-        <v>1095</v>
+        <v>616</v>
       </c>
       <c r="F2" t="n">
-        <v>1318</v>
+        <v>179</v>
       </c>
       <c r="G2" t="n">
-        <v>334</v>
+        <v>9</v>
       </c>
       <c r="H2" t="n">
-        <v>835</v>
+        <v>375</v>
       </c>
       <c r="I2" t="n">
-        <v>696</v>
+        <v>989</v>
       </c>
       <c r="J2" t="n">
-        <v>125</v>
+        <v>726</v>
       </c>
     </row>
   </sheetData>
@@ -616,72 +942,72 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>19770</v>
+        <v>18296</v>
       </c>
       <c r="B1" t="n">
-        <v>75</v>
+        <v>515</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>253</v>
+        <v>195</v>
       </c>
       <c r="B2" t="n">
-        <v>409</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>690</v>
+        <v>1379</v>
       </c>
       <c r="D2" t="n">
-        <v>781</v>
+        <v>597</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>1490</v>
+        <v>40</v>
       </c>
       <c r="G2" t="n">
-        <v>644</v>
+        <v>738</v>
       </c>
       <c r="H2" t="n">
-        <v>205</v>
+        <v>380</v>
       </c>
       <c r="I2" t="n">
-        <v>1553</v>
+        <v>1580</v>
       </c>
       <c r="J2" t="n">
-        <v>1121</v>
+        <v>972</v>
       </c>
       <c r="K2" t="n">
-        <v>1649</v>
+        <v>269</v>
       </c>
       <c r="L2" t="n">
-        <v>14</v>
+        <v>282</v>
       </c>
       <c r="M2" t="n">
-        <v>1331</v>
+        <v>569</v>
       </c>
       <c r="N2" t="n">
-        <v>370</v>
+        <v>1118</v>
       </c>
       <c r="O2" t="n">
-        <v>1021</v>
+        <v>872</v>
       </c>
       <c r="P2" t="n">
-        <v>312</v>
+        <v>1365</v>
       </c>
       <c r="Q2" t="n">
-        <v>118</v>
+        <v>489</v>
       </c>
       <c r="R2" t="n">
-        <v>1120</v>
+        <v>971</v>
       </c>
       <c r="S2" t="n">
-        <v>958</v>
+        <v>808</v>
       </c>
       <c r="T2" t="n">
-        <v>622</v>
+        <v>556</v>
       </c>
     </row>
   </sheetData>
@@ -700,10 +1026,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>20507</v>
+        <v>17814</v>
       </c>
       <c r="B1" t="n">
-        <v>125</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="2">
@@ -711,61 +1037,61 @@
         <v>7</v>
       </c>
       <c r="B2" t="n">
-        <v>1075</v>
+        <v>1446</v>
       </c>
       <c r="C2" t="n">
-        <v>1344</v>
+        <v>1146</v>
       </c>
       <c r="D2" t="n">
-        <v>1228</v>
+        <v>745</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>1638</v>
+        <v>1480</v>
       </c>
       <c r="G2" t="n">
-        <v>1651</v>
+        <v>299</v>
       </c>
       <c r="H2" t="n">
+        <v>211</v>
+      </c>
+      <c r="I2" t="n">
+        <v>647</v>
+      </c>
+      <c r="J2" t="n">
+        <v>924</v>
+      </c>
+      <c r="K2" t="n">
+        <v>78</v>
+      </c>
+      <c r="L2" t="n">
+        <v>113</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1306</v>
+      </c>
+      <c r="N2" t="n">
+        <v>632</v>
+      </c>
+      <c r="O2" t="n">
         <v>433</v>
       </c>
-      <c r="I2" t="n">
-        <v>825</v>
-      </c>
-      <c r="J2" t="n">
-        <v>170</v>
-      </c>
-      <c r="K2" t="n">
-        <v>660</v>
-      </c>
-      <c r="L2" t="n">
-        <v>531</v>
-      </c>
-      <c r="M2" t="n">
-        <v>1479</v>
-      </c>
-      <c r="N2" t="n">
-        <v>316</v>
-      </c>
-      <c r="O2" t="n">
-        <v>955</v>
-      </c>
       <c r="P2" t="n">
+        <v>1132</v>
+      </c>
+      <c r="Q2" t="n">
         <v>959</v>
       </c>
-      <c r="Q2" t="n">
-        <v>1271</v>
-      </c>
       <c r="R2" t="n">
-        <v>681</v>
+        <v>503</v>
       </c>
       <c r="S2" t="n">
-        <v>101</v>
+        <v>369</v>
       </c>
       <c r="T2" t="n">
-        <v>74</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -784,42 +1110,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>111153</v>
+        <v>108576</v>
       </c>
       <c r="B1" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8464</v>
+        <v>8190</v>
       </c>
       <c r="B2" t="n">
-        <v>1802</v>
+        <v>11970</v>
       </c>
       <c r="C2" t="n">
-        <v>11833</v>
+        <v>6135</v>
       </c>
       <c r="D2" t="n">
-        <v>2649</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>6331</v>
       </c>
       <c r="F2" t="n">
-        <v>4394</v>
+        <v>9468</v>
       </c>
       <c r="G2" t="n">
-        <v>4248</v>
+        <v>1223</v>
       </c>
       <c r="H2" t="n">
-        <v>10370</v>
+        <v>1228</v>
       </c>
       <c r="I2" t="n">
-        <v>9685</v>
+        <v>3812</v>
       </c>
       <c r="J2" t="n">
-        <v>4953</v>
+        <v>7464</v>
       </c>
     </row>
   </sheetData>
@@ -838,10 +1164,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="n">
-        <v>114471</v>
+        <v>98735</v>
       </c>
       <c r="B1" t="n">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr"/>
@@ -854,34 +1180,358 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>712</v>
+        <v>6527</v>
       </c>
       <c r="B2" t="n">
-        <v>2031</v>
+        <v>4350</v>
       </c>
       <c r="C2" t="n">
-        <v>848</v>
+        <v>4136</v>
       </c>
       <c r="D2" t="n">
-        <v>12861</v>
+        <v>11539</v>
       </c>
       <c r="E2" t="n">
-        <v>5089</v>
+        <v>2287</v>
       </c>
       <c r="F2" t="n">
-        <v>9463</v>
+        <v>7805</v>
       </c>
       <c r="G2" t="n">
-        <v>9091</v>
+        <v>22</v>
       </c>
       <c r="H2" t="n">
-        <v>7252</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>14369</v>
+        <v>8545</v>
       </c>
       <c r="J2" t="n">
+        <v>769</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CV2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>44170627</v>
+      </c>
+      <c r="B1" t="n">
+        <v>3614057</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>93049</v>
+      </c>
+      <c r="B2" t="n">
+        <v>137075</v>
+      </c>
+      <c r="C2" t="n">
         <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>777779</v>
+      </c>
+      <c r="E2" t="n">
+        <v>717998</v>
+      </c>
+      <c r="F2" t="n">
+        <v>643361</v>
+      </c>
+      <c r="G2" t="n">
+        <v>572657</v>
+      </c>
+      <c r="H2" t="n">
+        <v>115801</v>
+      </c>
+      <c r="I2" t="n">
+        <v>286687</v>
+      </c>
+      <c r="J2" t="n">
+        <v>128286</v>
+      </c>
+      <c r="K2" t="n">
+        <v>835870</v>
+      </c>
+      <c r="L2" t="n">
+        <v>603160</v>
+      </c>
+      <c r="M2" t="n">
+        <v>441546</v>
+      </c>
+      <c r="N2" t="n">
+        <v>464997</v>
+      </c>
+      <c r="O2" t="n">
+        <v>247699</v>
+      </c>
+      <c r="P2" t="n">
+        <v>39522</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>756278</v>
+      </c>
+      <c r="R2" t="n">
+        <v>146536</v>
+      </c>
+      <c r="S2" t="n">
+        <v>452832</v>
+      </c>
+      <c r="T2" t="n">
+        <v>215226</v>
+      </c>
+      <c r="U2" t="n">
+        <v>314637</v>
+      </c>
+      <c r="V2" t="n">
+        <v>633682</v>
+      </c>
+      <c r="W2" t="n">
+        <v>495376</v>
+      </c>
+      <c r="X2" t="n">
+        <v>391710</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>74457</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>197444</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>420857</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>116131</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>508217</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>699598</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>414795</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>513653</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>223351</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>347537</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>243465</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>365433</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>547781</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>591251</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>617095</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>378355</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>795986</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>6257</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>201983</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>851638</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>747878</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>26129</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>97412</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>232698</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>48502</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>261864</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>337397</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>348845</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>718632</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>301622</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>792733</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>175100</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>530627</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>701989</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>183477</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>40748</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>413710</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>115440</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>16634</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>167790</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>266109</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>510273</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>311153</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>426804</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>813230</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>283553</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>141997</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>261849</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>342061</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>666559</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>421655</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>572531</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>479513</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>667585</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>821935</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>741535</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>64163</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>690795</v>
+      </c>
+      <c r="CE2" t="n">
+        <v>623017</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>90206</v>
+      </c>
+      <c r="CG2" t="n">
+        <v>162845</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>750068</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>83086</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>2811</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>616698</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>290903</v>
+      </c>
+      <c r="CM2" t="n">
+        <v>558785</v>
+      </c>
+      <c r="CN2" t="n">
+        <v>452320</v>
+      </c>
+      <c r="CO2" t="n">
+        <v>230363</v>
+      </c>
+      <c r="CP2" t="n">
+        <v>58896</v>
+      </c>
+      <c r="CQ2" t="n">
+        <v>522382</v>
+      </c>
+      <c r="CR2" t="n">
+        <v>378181</v>
+      </c>
+      <c r="CS2" t="n">
+        <v>449524</v>
+      </c>
+      <c r="CT2" t="n">
+        <v>795894</v>
+      </c>
+      <c r="CU2" t="n">
+        <v>190432</v>
+      </c>
+      <c r="CV2" t="n">
+        <v>545973</v>
       </c>
     </row>
   </sheetData>

</xml_diff>